<commit_message>
Add TRI analysis results for Simulado III
Generate Item Response Theory (IRT) analysis outputs for 2nd and 3rd grade Portuguese and Math assessments. Includes new R scripts (Fit_3PL_Fix_2EM_MT_S3.R and Fit_3PL_Fix_3EM_LP_S3.R) adapted to estimate 3PL models with fixed parameters from SAEB calibration. Results include item characteristic curves, proficiency estimates, and fit statistics for 60+ items across three configurations (2EM_LP, 2EM_MT, 3EM_LP).
</commit_message>
<xml_diff>
--- a/Piaui/2026/Julho/Dados/gabarito_2serie_mt 3ª SIMULA.xlsx
+++ b/Piaui/2026/Julho/Dados/gabarito_2serie_mt 3ª SIMULA.xlsx
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="MT_2EM" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="MT_2EM_S3" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="60">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t xml:space="preserve">rpa_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sim</t>
   </si>
   <si>
     <t xml:space="preserve">rpa_005</t>
@@ -1280,12 +1283,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="8.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="2" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="35.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="2" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="35.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1293,24 +1296,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1318,475 +1318,383 @@
       <c r="A2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="D2" s="8"/>
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="13" t="s">
-        <v>10</v>
-      </c>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>12</v>
-      </c>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
+      <c r="B5" s="14" t="n">
+        <v>1.56</v>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1.56</v>
+        <v>2.673</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>2.673</v>
+        <v>0.031</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.031</v>
+        <v>383.669</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>383.669</v>
-      </c>
-      <c r="G5" s="14" t="n">
         <v>0.223</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>13</v>
+      <c r="G5" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>5.444</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>522.224</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>0.071</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>0.372</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>5.444</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>522.224</v>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>0.071</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>39</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0.843417332943628</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.843417332943628</v>
+        <v>1.01328778238753</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1.01328778238753</v>
+        <v>0.0168683466588725</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0168683466588725</v>
+        <v>300.664389119377</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>300.664389119377</v>
-      </c>
-      <c r="G7" s="2" t="n">
         <v>0.0161555405979066</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>15</v>
+      <c r="G7" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>16</v>
+        <v>40</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1.0627797687673</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1.0627797687673</v>
+        <v>3.25034579224713</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>3.25034579224713</v>
+        <v>0.0212555953753461</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.0212555953753461</v>
+        <v>412.517289612357</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>412.517289612357</v>
-      </c>
-      <c r="G8" s="2" t="n">
         <v>0.178081424286593</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>17</v>
+      <c r="G8" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>11</v>
+        <v>41</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1.44617244574152</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1.44617244574152</v>
+        <v>2.66265077769934</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2.66265077769934</v>
+        <v>0.0289234489148303</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.0289234489148303</v>
+        <v>383.132538884967</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>383.132538884967</v>
-      </c>
-      <c r="G9" s="2" t="n">
         <v>0.175890036350279</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>18</v>
+      <c r="G9" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>20</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="G11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>16</v>
+        <v>44</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1.70485770995118</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1.70485770995118</v>
+        <v>2.21387696226408</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2.21387696226408</v>
+        <v>0.0340971541990235</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0340971541990235</v>
+        <v>360.693848113204</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>360.693848113204</v>
-      </c>
-      <c r="G12" s="2" t="n">
         <v>0.174632413573961</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>21</v>
+      <c r="G12" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>8</v>
+        <v>45</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>1.24657501230464</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1.24657501230464</v>
+        <v>1.85487257458894</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1.85487257458894</v>
+        <v>0.0249315002460928</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0249315002460928</v>
+        <v>342.743628729447</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>342.743628729447</v>
-      </c>
-      <c r="G13" s="2" t="n">
         <v>0.103844749041497</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>22</v>
+      <c r="G13" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>19</v>
+        <v>46</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1.22742731801846</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.22742731801846</v>
+        <v>2.67255617837511</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2.67255617837511</v>
+        <v>0.0245485463603693</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0245485463603693</v>
+        <v>383.627808918756</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>383.627808918756</v>
-      </c>
-      <c r="G14" s="2" t="n">
         <v>0.193535074744008</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>23</v>
+      <c r="G14" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>11</v>
+        <v>47</v>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>1.663</v>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1.663</v>
+        <v>2.836</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>2.836</v>
+        <v>0.033</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.033</v>
+        <v>391.822</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>391.822</v>
-      </c>
-      <c r="G15" s="14" t="n">
         <v>0.22</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>24</v>
+      <c r="G15" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>11</v>
+        <v>48</v>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>2.867</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2.867</v>
+        <v>2.358</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>2.358</v>
+        <v>0.057</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.057</v>
+        <v>367.893</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>367.893</v>
-      </c>
-      <c r="G16" s="14" t="n">
         <v>0.156</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>25</v>
+      <c r="G16" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>26</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="G17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>8</v>
+        <v>51</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1.54104954143406</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.54104954143406</v>
+        <v>2.93556623650522</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>2.93556623650522</v>
+        <v>0.0308209908286812</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.0308209908286812</v>
+        <v>396.778311825261</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>396.778311825261</v>
-      </c>
-      <c r="G19" s="2" t="n">
         <v>0.109863312205395</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>27</v>
+      <c r="G19" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>11</v>
+        <v>52</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>2.61541934777186</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2.61541934777186</v>
+        <v>2.57156058184516</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>2.57156058184516</v>
+        <v>0.0523083869554372</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.0523083869554372</v>
+        <v>378.578029092258</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>378.578029092258</v>
-      </c>
-      <c r="G20" s="2" t="n">
         <v>0.214850619455008</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>28</v>
+      <c r="G20" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>19</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="13" t="s">
-        <v>29</v>
-      </c>
+      <c r="G21" s="13"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H22" s="13" t="s">
-        <v>30</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="G22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H23" s="13" t="s">
-        <v>31</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="G23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>2.3242653531958</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.3242653531958</v>
+        <v>2.81373560338526</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>2.81373560338526</v>
+        <v>0.046485307063916</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.046485307063916</v>
+        <v>390.686780169263</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>390.686780169263</v>
-      </c>
-      <c r="G27" s="2" t="n">
         <v>0.125612831543424</v>
       </c>
-      <c r="H27" s="2" t="s">
-        <v>32</v>
+      <c r="G27" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exclude items 7, 8 from 3EM_LP TRI calibration
Update TRI exclusion criteria for 3EM_LP to remove items 7 and 8 alongside item 5. All three items demonstrate weak discrimination and low point-biserial correlation; items 5 and 8 show evidence of stronger competing alternatives than the official answer key. Updates R script, Python reporting configuration, and regenerates all associated reports and results.
</commit_message>
<xml_diff>
--- a/Piaui/2026/Julho/Dados/gabarito_2serie_mt 3ª SIMULA.xlsx
+++ b/Piaui/2026/Julho/Dados/gabarito_2serie_mt 3ª SIMULA.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="60">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -1365,24 +1365,11 @@
       <c r="A6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="14" t="n">
-        <v>0.372</v>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>5.444</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>522.224</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>0.071</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">

</xml_diff>